<commit_message>
Parameter optimastion scripts for MStra with updated plots for new thresholds. Implemented Hanning window in ElderNet windows
</commit_message>
<xml_diff>
--- a/mstraczkiewicz/MStraPlots_FreeLiving/FreeLiving_MStra_Results.xlsx
+++ b/mstraczkiewicz/MStraPlots_FreeLiving/FreeLiving_MStra_Results.xlsx
@@ -8,6 +8,7 @@
   <sheets>
     <sheet name="All" sheetId="2" r:id="rId3"/>
     <sheet name="By_Subject" sheetId="3" r:id="rId5"/>
+    <sheet name="All_Files" sheetId="4" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
@@ -15,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="258" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="606" uniqueCount="32">
   <si>
     <t>Subject</t>
   </si>
@@ -99,6 +100,18 @@
   </si>
   <si>
     <t>mean_F1</t>
+  </si>
+  <si>
+    <t>sum_TP</t>
+  </si>
+  <si>
+    <t>sum_FP</t>
+  </si>
+  <si>
+    <t>sum_TN</t>
+  </si>
+  <si>
+    <t>sum_FN</t>
   </si>
 </sst>
 </file>
@@ -599,15 +612,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.88671875" customWidth="true"/>
     <col min="2" max="2" width="10.88671875" customWidth="true"/>
-    <col min="3" max="3" width="13.88671875" customWidth="true"/>
-    <col min="4" max="4" width="13.88671875" customWidth="true"/>
-    <col min="5" max="5" width="13.5546875" customWidth="true"/>
-    <col min="6" max="6" width="13.5546875" customWidth="true"/>
+    <col min="3" max="3" width="7.33203125" customWidth="true"/>
+    <col min="4" max="4" width="7.21875" customWidth="true"/>
+    <col min="5" max="5" width="7.6640625" customWidth="true"/>
+    <col min="6" max="6" width="7.5546875" customWidth="true"/>
+    <col min="7" max="7" width="13.5546875" customWidth="true"/>
+    <col min="8" max="8" width="13.5546875" customWidth="true"/>
+    <col min="9" max="9" width="12.5546875" customWidth="true"/>
+    <col min="10" max="10" width="13.5546875" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -618,16 +635,28 @@
         <v>23</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>27</v>
+        <v>31</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="2">
@@ -638,15 +667,27 @@
         <v>1</v>
       </c>
       <c r="C2" s="0">
+        <v>1740</v>
+      </c>
+      <c r="D2" s="0">
+        <v>2510</v>
+      </c>
+      <c r="E2" s="0">
+        <v>6586</v>
+      </c>
+      <c r="F2" s="0">
+        <v>1365</v>
+      </c>
+      <c r="G2" s="0">
+        <v>0.40941176470588236</v>
+      </c>
+      <c r="H2" s="0">
+        <v>0.56038647342995174</v>
+      </c>
+      <c r="I2" s="0">
         <v>0.6824030817146135</v>
       </c>
-      <c r="D2" s="0">
-        <v>0.40941176470588236</v>
-      </c>
-      <c r="E2" s="0">
-        <v>0.56038647342995174</v>
-      </c>
-      <c r="F2" s="0">
+      <c r="J2" s="0">
         <v>0.47314751869476551</v>
       </c>
     </row>
@@ -658,15 +699,27 @@
         <v>1</v>
       </c>
       <c r="C3" s="0">
+        <v>250</v>
+      </c>
+      <c r="D3" s="0">
+        <v>1500</v>
+      </c>
+      <c r="E3" s="0">
+        <v>20336</v>
+      </c>
+      <c r="F3" s="0">
+        <v>600</v>
+      </c>
+      <c r="G3" s="0">
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="H3" s="0">
+        <v>0.29411764705882354</v>
+      </c>
+      <c r="I3" s="0">
         <v>0.9074318963237239</v>
       </c>
-      <c r="D3" s="0">
-        <v>0.14285714285714285</v>
-      </c>
-      <c r="E3" s="0">
-        <v>0.29411764705882354</v>
-      </c>
-      <c r="F3" s="0">
+      <c r="J3" s="0">
         <v>0.19230769230769229</v>
       </c>
     </row>
@@ -678,15 +731,27 @@
         <v>1</v>
       </c>
       <c r="C4" s="0">
+        <v>130</v>
+      </c>
+      <c r="D4" s="0">
+        <v>1770</v>
+      </c>
+      <c r="E4" s="0">
+        <v>11606</v>
+      </c>
+      <c r="F4" s="0">
+        <v>2270</v>
+      </c>
+      <c r="G4" s="0">
+        <v>0.068421052631578952</v>
+      </c>
+      <c r="H4" s="0">
+        <v>0.054166666666666669</v>
+      </c>
+      <c r="I4" s="0">
         <v>0.74391480730223125</v>
       </c>
-      <c r="D4" s="0">
-        <v>0.068421052631578952</v>
-      </c>
-      <c r="E4" s="0">
-        <v>0.054166666666666669</v>
-      </c>
-      <c r="F4" s="0">
+      <c r="J4" s="0">
         <v>0.060465116279069767</v>
       </c>
     </row>
@@ -698,15 +763,27 @@
         <v>1</v>
       </c>
       <c r="C5" s="0">
+        <v>609</v>
+      </c>
+      <c r="D5" s="0">
+        <v>1441</v>
+      </c>
+      <c r="E5" s="0">
+        <v>9193</v>
+      </c>
+      <c r="F5" s="0">
+        <v>1771</v>
+      </c>
+      <c r="G5" s="0">
+        <v>0.2970731707317073</v>
+      </c>
+      <c r="H5" s="0">
+        <v>0.25588235294117645</v>
+      </c>
+      <c r="I5" s="0">
         <v>0.75318887352082375</v>
       </c>
-      <c r="D5" s="0">
-        <v>0.2970731707317073</v>
-      </c>
-      <c r="E5" s="0">
-        <v>0.25588235294117645</v>
-      </c>
-      <c r="F5" s="0">
+      <c r="J5" s="0">
         <v>0.27494356659142211</v>
       </c>
     </row>
@@ -718,15 +795,27 @@
         <v>1</v>
       </c>
       <c r="C6" s="0">
+        <v>435</v>
+      </c>
+      <c r="D6" s="0">
+        <v>3665</v>
+      </c>
+      <c r="E6" s="0">
+        <v>10706</v>
+      </c>
+      <c r="F6" s="0">
+        <v>690</v>
+      </c>
+      <c r="G6" s="0">
+        <v>0.10609756097560975</v>
+      </c>
+      <c r="H6" s="0">
+        <v>0.38666666666666666</v>
+      </c>
+      <c r="I6" s="0">
         <v>0.71895973154362414</v>
       </c>
-      <c r="D6" s="0">
-        <v>0.10609756097560975</v>
-      </c>
-      <c r="E6" s="0">
-        <v>0.38666666666666666</v>
-      </c>
-      <c r="F6" s="0">
+      <c r="J6" s="0">
         <v>0.1665071770334928</v>
       </c>
     </row>
@@ -738,15 +827,27 @@
         <v>1</v>
       </c>
       <c r="C7" s="0">
+        <v>1345</v>
+      </c>
+      <c r="D7" s="0">
+        <v>6355</v>
+      </c>
+      <c r="E7" s="0">
+        <v>12221</v>
+      </c>
+      <c r="F7" s="0">
+        <v>4250</v>
+      </c>
+      <c r="G7" s="0">
+        <v>0.17467532467532468</v>
+      </c>
+      <c r="H7" s="0">
+        <v>0.24039320822162646</v>
+      </c>
+      <c r="I7" s="0">
         <v>0.56125108601216334</v>
       </c>
-      <c r="D7" s="0">
-        <v>0.17467532467532468</v>
-      </c>
-      <c r="E7" s="0">
-        <v>0.24039320822162646</v>
-      </c>
-      <c r="F7" s="0">
+      <c r="J7" s="0">
         <v>0.202331703647988</v>
       </c>
     </row>
@@ -758,15 +859,27 @@
         <v>1</v>
       </c>
       <c r="C8" s="0">
+        <v>100</v>
+      </c>
+      <c r="D8" s="0">
+        <v>2650</v>
+      </c>
+      <c r="E8" s="0">
+        <v>17501</v>
+      </c>
+      <c r="F8" s="0">
+        <v>1450</v>
+      </c>
+      <c r="G8" s="0">
+        <v>0.036363636363636362</v>
+      </c>
+      <c r="H8" s="0">
+        <v>0.064516129032258063</v>
+      </c>
+      <c r="I8" s="0">
         <v>0.81106861434956912</v>
       </c>
-      <c r="D8" s="0">
-        <v>0.036363636363636362</v>
-      </c>
-      <c r="E8" s="0">
-        <v>0.064516129032258063</v>
-      </c>
-      <c r="F8" s="0">
+      <c r="J8" s="0">
         <v>0.046511627906976744</v>
       </c>
     </row>
@@ -778,15 +891,27 @@
         <v>1</v>
       </c>
       <c r="C9" s="0">
+        <v>0</v>
+      </c>
+      <c r="D9" s="0">
+        <v>250</v>
+      </c>
+      <c r="E9" s="0">
+        <v>21284</v>
+      </c>
+      <c r="F9" s="0">
+        <v>1405</v>
+      </c>
+      <c r="G9" s="0">
+        <v>0</v>
+      </c>
+      <c r="H9" s="0">
+        <v>0</v>
+      </c>
+      <c r="I9" s="0">
         <v>0.9278521295610096</v>
       </c>
-      <c r="D9" s="0">
-        <v>0</v>
-      </c>
-      <c r="E9" s="0">
-        <v>0</v>
-      </c>
-      <c r="F9" s="0">
+      <c r="J9" s="0">
         <v>0</v>
       </c>
     </row>
@@ -798,15 +923,27 @@
         <v>1</v>
       </c>
       <c r="C10" s="0">
+        <v>91</v>
+      </c>
+      <c r="D10" s="0">
+        <v>1009</v>
+      </c>
+      <c r="E10" s="0">
+        <v>15438</v>
+      </c>
+      <c r="F10" s="0">
+        <v>1294</v>
+      </c>
+      <c r="G10" s="0">
+        <v>0.082727272727272733</v>
+      </c>
+      <c r="H10" s="0">
+        <v>0.065703971119133578</v>
+      </c>
+      <c r="I10" s="0">
         <v>0.8708501570210857</v>
       </c>
-      <c r="D10" s="0">
-        <v>0.082727272727272733</v>
-      </c>
-      <c r="E10" s="0">
-        <v>0.065703971119133578</v>
-      </c>
-      <c r="F10" s="0">
+      <c r="J10" s="0">
         <v>0.073239436619718309</v>
       </c>
     </row>
@@ -818,15 +955,27 @@
         <v>1</v>
       </c>
       <c r="C11" s="0">
+        <v>330</v>
+      </c>
+      <c r="D11" s="0">
+        <v>920</v>
+      </c>
+      <c r="E11" s="0">
+        <v>8676</v>
+      </c>
+      <c r="F11" s="0">
+        <v>900</v>
+      </c>
+      <c r="G11" s="0">
+        <v>0.26400000000000001</v>
+      </c>
+      <c r="H11" s="0">
+        <v>0.26829268292682928</v>
+      </c>
+      <c r="I11" s="0">
         <v>0.83188619988915569</v>
       </c>
-      <c r="D11" s="0">
-        <v>0.26400000000000001</v>
-      </c>
-      <c r="E11" s="0">
-        <v>0.26829268292682928</v>
-      </c>
-      <c r="F11" s="0">
+      <c r="J11" s="0">
         <v>0.26612903225806456</v>
       </c>
     </row>
@@ -838,15 +987,27 @@
         <v>1</v>
       </c>
       <c r="C12" s="0">
+        <v>440</v>
+      </c>
+      <c r="D12" s="0">
+        <v>2860</v>
+      </c>
+      <c r="E12" s="0">
+        <v>9151</v>
+      </c>
+      <c r="F12" s="0">
+        <v>970</v>
+      </c>
+      <c r="G12" s="0">
+        <v>0.13333333333333333</v>
+      </c>
+      <c r="H12" s="0">
+        <v>0.31205673758865249</v>
+      </c>
+      <c r="I12" s="0">
         <v>0.71462633186796809</v>
       </c>
-      <c r="D12" s="0">
-        <v>0.13333333333333333</v>
-      </c>
-      <c r="E12" s="0">
-        <v>0.31205673758865249</v>
-      </c>
-      <c r="F12" s="0">
+      <c r="J12" s="0">
         <v>0.18683651804670912</v>
       </c>
     </row>
@@ -858,15 +1019,27 @@
         <v>1</v>
       </c>
       <c r="C13" s="0">
+        <v>0</v>
+      </c>
+      <c r="D13" s="0">
+        <v>1000</v>
+      </c>
+      <c r="E13" s="0">
+        <v>11753</v>
+      </c>
+      <c r="F13" s="0">
+        <v>1615</v>
+      </c>
+      <c r="G13" s="0">
+        <v>0</v>
+      </c>
+      <c r="H13" s="0">
+        <v>0</v>
+      </c>
+      <c r="I13" s="0">
         <v>0.81799832962138086</v>
       </c>
-      <c r="D13" s="0">
-        <v>0</v>
-      </c>
-      <c r="E13" s="0">
-        <v>0</v>
-      </c>
-      <c r="F13" s="0">
+      <c r="J13" s="0">
         <v>0</v>
       </c>
     </row>
@@ -878,15 +1051,27 @@
         <v>1</v>
       </c>
       <c r="C14" s="0">
+        <v>315</v>
+      </c>
+      <c r="D14" s="0">
+        <v>1485</v>
+      </c>
+      <c r="E14" s="0">
+        <v>6781</v>
+      </c>
+      <c r="F14" s="0">
+        <v>870</v>
+      </c>
+      <c r="G14" s="0">
+        <v>0.17499999999999999</v>
+      </c>
+      <c r="H14" s="0">
+        <v>0.26582278481012656</v>
+      </c>
+      <c r="I14" s="0">
         <v>0.75082001904560369</v>
       </c>
-      <c r="D14" s="0">
-        <v>0.17499999999999999</v>
-      </c>
-      <c r="E14" s="0">
-        <v>0.26582278481012656</v>
-      </c>
-      <c r="F14" s="0">
+      <c r="J14" s="0">
         <v>0.21105527638190952</v>
       </c>
     </row>
@@ -898,7 +1083,465 @@
         <v>1</v>
       </c>
       <c r="C15" s="0">
+        <v>475</v>
+      </c>
+      <c r="D15" s="0">
+        <v>1125</v>
+      </c>
+      <c r="E15" s="0">
+        <v>5516</v>
+      </c>
+      <c r="F15" s="0">
+        <v>645</v>
+      </c>
+      <c r="G15" s="0">
+        <v>0.296875</v>
+      </c>
+      <c r="H15" s="0">
+        <v>0.42410714285714285</v>
+      </c>
+      <c r="I15" s="0">
         <v>0.7719366061074604</v>
+      </c>
+      <c r="J15" s="0">
+        <v>0.34926470588235292</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="6.88671875" customWidth="true"/>
+    <col min="2" max="2" width="12.5546875" customWidth="true"/>
+    <col min="3" max="3" width="13.5546875" customWidth="true"/>
+    <col min="4" max="4" width="13.5546875" customWidth="true"/>
+    <col min="5" max="5" width="13.5546875" customWidth="true"/>
+    <col min="6" max="6" width="5" customWidth="true"/>
+    <col min="7" max="7" width="6" customWidth="true"/>
+    <col min="8" max="8" width="5" customWidth="true"/>
+    <col min="9" max="9" width="5" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>0.9074318963237239</v>
+      </c>
+      <c r="C2" s="0">
+        <v>0.19230769230769229</v>
+      </c>
+      <c r="D2" s="0">
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="E2" s="0">
+        <v>0.29411764705882354</v>
+      </c>
+      <c r="F2" s="0">
+        <v>250</v>
+      </c>
+      <c r="G2" s="0">
+        <v>20336</v>
+      </c>
+      <c r="H2" s="0">
+        <v>1500</v>
+      </c>
+      <c r="I2" s="0">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0">
+        <v>0.74391480730223125</v>
+      </c>
+      <c r="C3" s="0">
+        <v>0.060465116279069767</v>
+      </c>
+      <c r="D3" s="0">
+        <v>0.068421052631578952</v>
+      </c>
+      <c r="E3" s="0">
+        <v>0.054166666666666669</v>
+      </c>
+      <c r="F3" s="0">
+        <v>130</v>
+      </c>
+      <c r="G3" s="0">
+        <v>11606</v>
+      </c>
+      <c r="H3" s="0">
+        <v>1770</v>
+      </c>
+      <c r="I3" s="0">
+        <v>2270</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0">
+        <v>0.75318887352082375</v>
+      </c>
+      <c r="C4" s="0">
+        <v>0.27494356659142211</v>
+      </c>
+      <c r="D4" s="0">
+        <v>0.2970731707317073</v>
+      </c>
+      <c r="E4" s="0">
+        <v>0.25588235294117645</v>
+      </c>
+      <c r="F4" s="0">
+        <v>609</v>
+      </c>
+      <c r="G4" s="0">
+        <v>9193</v>
+      </c>
+      <c r="H4" s="0">
+        <v>1441</v>
+      </c>
+      <c r="I4" s="0">
+        <v>1771</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0">
+        <v>0.71895973154362414</v>
+      </c>
+      <c r="C5" s="0">
+        <v>0.1665071770334928</v>
+      </c>
+      <c r="D5" s="0">
+        <v>0.10609756097560975</v>
+      </c>
+      <c r="E5" s="0">
+        <v>0.38666666666666666</v>
+      </c>
+      <c r="F5" s="0">
+        <v>435</v>
+      </c>
+      <c r="G5" s="0">
+        <v>10706</v>
+      </c>
+      <c r="H5" s="0">
+        <v>3665</v>
+      </c>
+      <c r="I5" s="0">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0">
+        <v>0.56125108601216334</v>
+      </c>
+      <c r="C6" s="0">
+        <v>0.202331703647988</v>
+      </c>
+      <c r="D6" s="0">
+        <v>0.17467532467532468</v>
+      </c>
+      <c r="E6" s="0">
+        <v>0.24039320822162646</v>
+      </c>
+      <c r="F6" s="0">
+        <v>1345</v>
+      </c>
+      <c r="G6" s="0">
+        <v>12221</v>
+      </c>
+      <c r="H6" s="0">
+        <v>6355</v>
+      </c>
+      <c r="I6" s="0">
+        <v>4250</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0">
+        <v>0.6824030817146135</v>
+      </c>
+      <c r="C7" s="0">
+        <v>0.47314751869476551</v>
+      </c>
+      <c r="D7" s="0">
+        <v>0.40941176470588236</v>
+      </c>
+      <c r="E7" s="0">
+        <v>0.56038647342995174</v>
+      </c>
+      <c r="F7" s="0">
+        <v>1740</v>
+      </c>
+      <c r="G7" s="0">
+        <v>6586</v>
+      </c>
+      <c r="H7" s="0">
+        <v>2510</v>
+      </c>
+      <c r="I7" s="0">
+        <v>1365</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0">
+        <v>0.81106861434956912</v>
+      </c>
+      <c r="C8" s="0">
+        <v>0.046511627906976744</v>
+      </c>
+      <c r="D8" s="0">
+        <v>0.036363636363636362</v>
+      </c>
+      <c r="E8" s="0">
+        <v>0.064516129032258063</v>
+      </c>
+      <c r="F8" s="0">
+        <v>100</v>
+      </c>
+      <c r="G8" s="0">
+        <v>17501</v>
+      </c>
+      <c r="H8" s="0">
+        <v>2650</v>
+      </c>
+      <c r="I8" s="0">
+        <v>1450</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0">
+        <v>0.9278521295610096</v>
+      </c>
+      <c r="C9" s="0">
+        <v>0</v>
+      </c>
+      <c r="D9" s="0">
+        <v>0</v>
+      </c>
+      <c r="E9" s="0">
+        <v>0</v>
+      </c>
+      <c r="F9" s="0">
+        <v>0</v>
+      </c>
+      <c r="G9" s="0">
+        <v>21284</v>
+      </c>
+      <c r="H9" s="0">
+        <v>250</v>
+      </c>
+      <c r="I9" s="0">
+        <v>1405</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0">
+        <v>0.8708501570210857</v>
+      </c>
+      <c r="C10" s="0">
+        <v>0.073239436619718309</v>
+      </c>
+      <c r="D10" s="0">
+        <v>0.082727272727272733</v>
+      </c>
+      <c r="E10" s="0">
+        <v>0.065703971119133578</v>
+      </c>
+      <c r="F10" s="0">
+        <v>91</v>
+      </c>
+      <c r="G10" s="0">
+        <v>15438</v>
+      </c>
+      <c r="H10" s="0">
+        <v>1009</v>
+      </c>
+      <c r="I10" s="0">
+        <v>1294</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0">
+        <v>0.83188619988915569</v>
+      </c>
+      <c r="C11" s="0">
+        <v>0.26612903225806456</v>
+      </c>
+      <c r="D11" s="0">
+        <v>0.26400000000000001</v>
+      </c>
+      <c r="E11" s="0">
+        <v>0.26829268292682928</v>
+      </c>
+      <c r="F11" s="0">
+        <v>330</v>
+      </c>
+      <c r="G11" s="0">
+        <v>8676</v>
+      </c>
+      <c r="H11" s="0">
+        <v>920</v>
+      </c>
+      <c r="I11" s="0">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0">
+        <v>0.71462633186796809</v>
+      </c>
+      <c r="C12" s="0">
+        <v>0.18683651804670912</v>
+      </c>
+      <c r="D12" s="0">
+        <v>0.13333333333333333</v>
+      </c>
+      <c r="E12" s="0">
+        <v>0.31205673758865249</v>
+      </c>
+      <c r="F12" s="0">
+        <v>440</v>
+      </c>
+      <c r="G12" s="0">
+        <v>9151</v>
+      </c>
+      <c r="H12" s="0">
+        <v>2860</v>
+      </c>
+      <c r="I12" s="0">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0">
+        <v>0.81799832962138086</v>
+      </c>
+      <c r="C13" s="0">
+        <v>0</v>
+      </c>
+      <c r="D13" s="0">
+        <v>0</v>
+      </c>
+      <c r="E13" s="0">
+        <v>0</v>
+      </c>
+      <c r="F13" s="0">
+        <v>0</v>
+      </c>
+      <c r="G13" s="0">
+        <v>11753</v>
+      </c>
+      <c r="H13" s="0">
+        <v>1000</v>
+      </c>
+      <c r="I13" s="0">
+        <v>1615</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0">
+        <v>0.75082001904560369</v>
+      </c>
+      <c r="C14" s="0">
+        <v>0.21105527638190952</v>
+      </c>
+      <c r="D14" s="0">
+        <v>0.17499999999999999</v>
+      </c>
+      <c r="E14" s="0">
+        <v>0.26582278481012656</v>
+      </c>
+      <c r="F14" s="0">
+        <v>315</v>
+      </c>
+      <c r="G14" s="0">
+        <v>6781</v>
+      </c>
+      <c r="H14" s="0">
+        <v>1485</v>
+      </c>
+      <c r="I14" s="0">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0">
+        <v>0.7719366061074604</v>
+      </c>
+      <c r="C15" s="0">
+        <v>0.34926470588235292</v>
       </c>
       <c r="D15" s="0">
         <v>0.296875</v>
@@ -907,7 +1550,16 @@
         <v>0.42410714285714285</v>
       </c>
       <c r="F15" s="0">
-        <v>0.34926470588235292</v>
+        <v>475</v>
+      </c>
+      <c r="G15" s="0">
+        <v>5516</v>
+      </c>
+      <c r="H15" s="0">
+        <v>1125</v>
+      </c>
+      <c r="I15" s="0">
+        <v>645</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Mstra to remove faulty data including in plots and metric calculations. Added additional printouts showing quantity of faulty data
</commit_message>
<xml_diff>
--- a/mstraczkiewicz/MStraPlots_FreeLiving/FreeLiving_MStra_Results.xlsx
+++ b/mstraczkiewicz/MStraPlots_FreeLiving/FreeLiving_MStra_Results.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="606" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="841" uniqueCount="32">
   <si>
     <t>Subject</t>
   </si>
@@ -621,10 +621,10 @@
     <col min="4" max="4" width="7.21875" customWidth="true"/>
     <col min="5" max="5" width="7.6640625" customWidth="true"/>
     <col min="6" max="6" width="7.5546875" customWidth="true"/>
-    <col min="7" max="7" width="13.5546875" customWidth="true"/>
-    <col min="8" max="8" width="13.5546875" customWidth="true"/>
+    <col min="7" max="7" width="12.5546875" customWidth="true"/>
+    <col min="8" max="8" width="12.5546875" customWidth="true"/>
     <col min="9" max="9" width="12.5546875" customWidth="true"/>
-    <col min="10" max="10" width="13.5546875" customWidth="true"/>
+    <col min="10" max="10" width="12.5546875" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -667,28 +667,28 @@
         <v>1</v>
       </c>
       <c r="C2" s="0">
-        <v>1740</v>
+        <v>1425</v>
       </c>
       <c r="D2" s="0">
-        <v>2510</v>
+        <v>2575</v>
       </c>
       <c r="E2" s="0">
-        <v>6586</v>
+        <v>6521</v>
       </c>
       <c r="F2" s="0">
-        <v>1365</v>
+        <v>1680</v>
       </c>
       <c r="G2" s="0">
-        <v>0.40941176470588236</v>
+        <v>0.35625000000000001</v>
       </c>
       <c r="H2" s="0">
-        <v>0.56038647342995174</v>
+        <v>0.45893719806763283</v>
       </c>
       <c r="I2" s="0">
-        <v>0.6824030817146135</v>
+        <v>0.65125809359888531</v>
       </c>
       <c r="J2" s="0">
-        <v>0.47314751869476551</v>
+        <v>0.40112596762843067</v>
       </c>
     </row>
     <row r="3">
@@ -699,28 +699,28 @@
         <v>1</v>
       </c>
       <c r="C3" s="0">
-        <v>250</v>
+        <v>665</v>
       </c>
       <c r="D3" s="0">
-        <v>1500</v>
+        <v>4185</v>
       </c>
       <c r="E3" s="0">
-        <v>20336</v>
+        <v>17651</v>
       </c>
       <c r="F3" s="0">
-        <v>600</v>
+        <v>185</v>
       </c>
       <c r="G3" s="0">
-        <v>0.14285714285714285</v>
+        <v>0.13711340206185568</v>
       </c>
       <c r="H3" s="0">
-        <v>0.29411764705882354</v>
+        <v>0.78235294117647058</v>
       </c>
       <c r="I3" s="0">
-        <v>0.9074318963237239</v>
+        <v>0.80737018425460638</v>
       </c>
       <c r="J3" s="0">
-        <v>0.19230769230769229</v>
+        <v>0.23333333333333334</v>
       </c>
     </row>
     <row r="4">
@@ -731,28 +731,28 @@
         <v>1</v>
       </c>
       <c r="C4" s="0">
-        <v>130</v>
+        <v>1795</v>
       </c>
       <c r="D4" s="0">
-        <v>1770</v>
+        <v>3705</v>
       </c>
       <c r="E4" s="0">
-        <v>11606</v>
+        <v>9671</v>
       </c>
       <c r="F4" s="0">
-        <v>2270</v>
+        <v>605</v>
       </c>
       <c r="G4" s="0">
-        <v>0.068421052631578952</v>
+        <v>0.32636363636363636</v>
       </c>
       <c r="H4" s="0">
-        <v>0.054166666666666669</v>
+        <v>0.74791666666666667</v>
       </c>
       <c r="I4" s="0">
-        <v>0.74391480730223125</v>
+        <v>0.72680020283975655</v>
       </c>
       <c r="J4" s="0">
-        <v>0.060465116279069767</v>
+        <v>0.45443037974683548</v>
       </c>
     </row>
     <row r="5">
@@ -763,28 +763,28 @@
         <v>1</v>
       </c>
       <c r="C5" s="0">
-        <v>609</v>
+        <v>1697</v>
       </c>
       <c r="D5" s="0">
-        <v>1441</v>
+        <v>3303</v>
       </c>
       <c r="E5" s="0">
-        <v>9193</v>
+        <v>7331</v>
       </c>
       <c r="F5" s="0">
-        <v>1771</v>
+        <v>683</v>
       </c>
       <c r="G5" s="0">
-        <v>0.2970731707317073</v>
+        <v>0.33939999999999998</v>
       </c>
       <c r="H5" s="0">
-        <v>0.25588235294117645</v>
+        <v>0.71302521008403363</v>
       </c>
       <c r="I5" s="0">
-        <v>0.75318887352082375</v>
+        <v>0.69371446134931614</v>
       </c>
       <c r="J5" s="0">
-        <v>0.27494356659142211</v>
+        <v>0.45989159891598913</v>
       </c>
     </row>
     <row r="6">
@@ -795,28 +795,28 @@
         <v>1</v>
       </c>
       <c r="C6" s="0">
-        <v>435</v>
+        <v>385</v>
       </c>
       <c r="D6" s="0">
-        <v>3665</v>
+        <v>2015</v>
       </c>
       <c r="E6" s="0">
-        <v>10706</v>
+        <v>12356</v>
       </c>
       <c r="F6" s="0">
-        <v>690</v>
+        <v>740</v>
       </c>
       <c r="G6" s="0">
-        <v>0.10609756097560975</v>
+        <v>0.16041666666666668</v>
       </c>
       <c r="H6" s="0">
-        <v>0.38666666666666666</v>
+        <v>0.34222222222222221</v>
       </c>
       <c r="I6" s="0">
-        <v>0.71895973154362414</v>
+        <v>0.822212183789365</v>
       </c>
       <c r="J6" s="0">
-        <v>0.1665071770334928</v>
+        <v>0.21843971631205675</v>
       </c>
     </row>
     <row r="7">
@@ -827,28 +827,28 @@
         <v>1</v>
       </c>
       <c r="C7" s="0">
-        <v>1345</v>
+        <v>3750</v>
       </c>
       <c r="D7" s="0">
-        <v>6355</v>
+        <v>7400</v>
       </c>
       <c r="E7" s="0">
-        <v>12221</v>
+        <v>11176</v>
       </c>
       <c r="F7" s="0">
-        <v>4250</v>
+        <v>1845</v>
       </c>
       <c r="G7" s="0">
-        <v>0.17467532467532468</v>
+        <v>0.33632286995515698</v>
       </c>
       <c r="H7" s="0">
-        <v>0.24039320822162646</v>
+        <v>0.67024128686327078</v>
       </c>
       <c r="I7" s="0">
-        <v>0.56125108601216334</v>
+        <v>0.61751685904596421</v>
       </c>
       <c r="J7" s="0">
-        <v>0.202331703647988</v>
+        <v>0.44789489399820842</v>
       </c>
     </row>
     <row r="8">
@@ -859,28 +859,28 @@
         <v>1</v>
       </c>
       <c r="C8" s="0">
-        <v>100</v>
+        <v>415</v>
       </c>
       <c r="D8" s="0">
-        <v>2650</v>
+        <v>1335</v>
       </c>
       <c r="E8" s="0">
-        <v>17501</v>
+        <v>18816</v>
       </c>
       <c r="F8" s="0">
-        <v>1450</v>
+        <v>1135</v>
       </c>
       <c r="G8" s="0">
-        <v>0.036363636363636362</v>
+        <v>0.23714285714285716</v>
       </c>
       <c r="H8" s="0">
-        <v>0.064516129032258063</v>
+        <v>0.26774193548387099</v>
       </c>
       <c r="I8" s="0">
-        <v>0.81106861434956912</v>
+        <v>0.88618036035205749</v>
       </c>
       <c r="J8" s="0">
-        <v>0.046511627906976744</v>
+        <v>0.25151515151515152</v>
       </c>
     </row>
     <row r="9">
@@ -894,10 +894,10 @@
         <v>0</v>
       </c>
       <c r="D9" s="0">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="E9" s="0">
-        <v>21284</v>
+        <v>21334</v>
       </c>
       <c r="F9" s="0">
         <v>1405</v>
@@ -909,7 +909,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="0">
-        <v>0.9278521295610096</v>
+        <v>0.93003182353197611</v>
       </c>
       <c r="J9" s="0">
         <v>0</v>
@@ -923,28 +923,28 @@
         <v>1</v>
       </c>
       <c r="C10" s="0">
-        <v>91</v>
+        <v>985</v>
       </c>
       <c r="D10" s="0">
-        <v>1009</v>
+        <v>1415</v>
       </c>
       <c r="E10" s="0">
-        <v>15438</v>
+        <v>15032</v>
       </c>
       <c r="F10" s="0">
-        <v>1294</v>
+        <v>400</v>
       </c>
       <c r="G10" s="0">
-        <v>0.082727272727272733</v>
+        <v>0.41041666666666665</v>
       </c>
       <c r="H10" s="0">
-        <v>0.065703971119133578</v>
+        <v>0.71119133574007221</v>
       </c>
       <c r="I10" s="0">
-        <v>0.8708501570210857</v>
+        <v>0.89821668909825036</v>
       </c>
       <c r="J10" s="0">
-        <v>0.073239436619718309</v>
+        <v>0.52047556142668427</v>
       </c>
     </row>
     <row r="11">
@@ -955,28 +955,28 @@
         <v>1</v>
       </c>
       <c r="C11" s="0">
-        <v>330</v>
+        <v>355</v>
       </c>
       <c r="D11" s="0">
-        <v>920</v>
+        <v>1045</v>
       </c>
       <c r="E11" s="0">
-        <v>8676</v>
+        <v>8551</v>
       </c>
       <c r="F11" s="0">
-        <v>900</v>
+        <v>875</v>
       </c>
       <c r="G11" s="0">
-        <v>0.26400000000000001</v>
+        <v>0.25357142857142856</v>
       </c>
       <c r="H11" s="0">
-        <v>0.26829268292682928</v>
+        <v>0.2886178861788618</v>
       </c>
       <c r="I11" s="0">
-        <v>0.83188619988915569</v>
+        <v>0.82264917790504344</v>
       </c>
       <c r="J11" s="0">
-        <v>0.26612903225806456</v>
+        <v>0.26996197718631182</v>
       </c>
     </row>
     <row r="12">
@@ -987,28 +987,28 @@
         <v>1</v>
       </c>
       <c r="C12" s="0">
-        <v>440</v>
+        <v>540</v>
       </c>
       <c r="D12" s="0">
-        <v>2860</v>
+        <v>3710</v>
       </c>
       <c r="E12" s="0">
-        <v>9151</v>
+        <v>8301</v>
       </c>
       <c r="F12" s="0">
-        <v>970</v>
+        <v>870</v>
       </c>
       <c r="G12" s="0">
-        <v>0.13333333333333333</v>
+        <v>0.12705882352941175</v>
       </c>
       <c r="H12" s="0">
-        <v>0.31205673758865249</v>
+        <v>0.38297872340425532</v>
       </c>
       <c r="I12" s="0">
-        <v>0.71462633186796809</v>
+        <v>0.6587437597794501</v>
       </c>
       <c r="J12" s="0">
-        <v>0.18683651804670912</v>
+        <v>0.19081272084805651</v>
       </c>
     </row>
     <row r="13">
@@ -1019,28 +1019,28 @@
         <v>1</v>
       </c>
       <c r="C13" s="0">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="D13" s="0">
-        <v>1000</v>
+        <v>1283</v>
       </c>
       <c r="E13" s="0">
-        <v>11753</v>
+        <v>11470</v>
       </c>
       <c r="F13" s="0">
-        <v>1615</v>
+        <v>1448</v>
       </c>
       <c r="G13" s="0">
-        <v>0</v>
+        <v>0.11517241379310345</v>
       </c>
       <c r="H13" s="0">
-        <v>0</v>
+        <v>0.10340557275541795</v>
       </c>
       <c r="I13" s="0">
-        <v>0.81799832962138086</v>
+        <v>0.80992483296213813</v>
       </c>
       <c r="J13" s="0">
-        <v>0</v>
+        <v>0.10897226753670472</v>
       </c>
     </row>
     <row r="14">
@@ -1051,28 +1051,28 @@
         <v>1</v>
       </c>
       <c r="C14" s="0">
-        <v>315</v>
+        <v>605</v>
       </c>
       <c r="D14" s="0">
-        <v>1485</v>
+        <v>2445</v>
       </c>
       <c r="E14" s="0">
-        <v>6781</v>
+        <v>5821</v>
       </c>
       <c r="F14" s="0">
-        <v>870</v>
+        <v>580</v>
       </c>
       <c r="G14" s="0">
-        <v>0.17499999999999999</v>
+        <v>0.19836065573770492</v>
       </c>
       <c r="H14" s="0">
-        <v>0.26582278481012656</v>
+        <v>0.51054852320675104</v>
       </c>
       <c r="I14" s="0">
-        <v>0.75082001904560369</v>
+        <v>0.67992804994180511</v>
       </c>
       <c r="J14" s="0">
-        <v>0.21105527638190952</v>
+        <v>0.28571428571428575</v>
       </c>
     </row>
     <row r="15">
@@ -1083,28 +1083,28 @@
         <v>1</v>
       </c>
       <c r="C15" s="0">
-        <v>475</v>
+        <v>300</v>
       </c>
       <c r="D15" s="0">
-        <v>1125</v>
+        <v>1900</v>
       </c>
       <c r="E15" s="0">
-        <v>5516</v>
+        <v>4741</v>
       </c>
       <c r="F15" s="0">
-        <v>645</v>
+        <v>820</v>
       </c>
       <c r="G15" s="0">
-        <v>0.296875</v>
+        <v>0.13636363636363635</v>
       </c>
       <c r="H15" s="0">
-        <v>0.42410714285714285</v>
+        <v>0.26785714285714285</v>
       </c>
       <c r="I15" s="0">
-        <v>0.7719366061074604</v>
+        <v>0.64952969978095609</v>
       </c>
       <c r="J15" s="0">
-        <v>0.34926470588235292</v>
+        <v>0.18072289156626506</v>
       </c>
     </row>
   </sheetData>
@@ -1118,9 +1118,9 @@
   <cols>
     <col min="1" max="1" width="6.88671875" customWidth="true"/>
     <col min="2" max="2" width="12.5546875" customWidth="true"/>
-    <col min="3" max="3" width="13.5546875" customWidth="true"/>
-    <col min="4" max="4" width="13.5546875" customWidth="true"/>
-    <col min="5" max="5" width="13.5546875" customWidth="true"/>
+    <col min="3" max="3" width="12.5546875" customWidth="true"/>
+    <col min="4" max="4" width="12.5546875" customWidth="true"/>
+    <col min="5" max="5" width="12.5546875" customWidth="true"/>
     <col min="6" max="6" width="5" customWidth="true"/>
     <col min="7" max="7" width="6" customWidth="true"/>
     <col min="8" max="8" width="5" customWidth="true"/>
@@ -1161,28 +1161,28 @@
         <v>1</v>
       </c>
       <c r="B2" s="0">
-        <v>0.9074318963237239</v>
+        <v>0.80737018425460638</v>
       </c>
       <c r="C2" s="0">
-        <v>0.19230769230769229</v>
+        <v>0.23333333333333334</v>
       </c>
       <c r="D2" s="0">
-        <v>0.14285714285714285</v>
+        <v>0.13711340206185568</v>
       </c>
       <c r="E2" s="0">
-        <v>0.29411764705882354</v>
+        <v>0.78235294117647058</v>
       </c>
       <c r="F2" s="0">
-        <v>250</v>
+        <v>665</v>
       </c>
       <c r="G2" s="0">
-        <v>20336</v>
+        <v>17651</v>
       </c>
       <c r="H2" s="0">
-        <v>1500</v>
+        <v>4185</v>
       </c>
       <c r="I2" s="0">
-        <v>600</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3">
@@ -1190,28 +1190,28 @@
         <v>2</v>
       </c>
       <c r="B3" s="0">
-        <v>0.74391480730223125</v>
+        <v>0.72680020283975655</v>
       </c>
       <c r="C3" s="0">
-        <v>0.060465116279069767</v>
+        <v>0.45443037974683548</v>
       </c>
       <c r="D3" s="0">
-        <v>0.068421052631578952</v>
+        <v>0.32636363636363636</v>
       </c>
       <c r="E3" s="0">
-        <v>0.054166666666666669</v>
+        <v>0.74791666666666667</v>
       </c>
       <c r="F3" s="0">
-        <v>130</v>
+        <v>1795</v>
       </c>
       <c r="G3" s="0">
-        <v>11606</v>
+        <v>9671</v>
       </c>
       <c r="H3" s="0">
-        <v>1770</v>
+        <v>3705</v>
       </c>
       <c r="I3" s="0">
-        <v>2270</v>
+        <v>605</v>
       </c>
     </row>
     <row r="4">
@@ -1219,28 +1219,28 @@
         <v>3</v>
       </c>
       <c r="B4" s="0">
-        <v>0.75318887352082375</v>
+        <v>0.69371446134931614</v>
       </c>
       <c r="C4" s="0">
-        <v>0.27494356659142211</v>
+        <v>0.45989159891598913</v>
       </c>
       <c r="D4" s="0">
-        <v>0.2970731707317073</v>
+        <v>0.33939999999999998</v>
       </c>
       <c r="E4" s="0">
-        <v>0.25588235294117645</v>
+        <v>0.71302521008403363</v>
       </c>
       <c r="F4" s="0">
-        <v>609</v>
+        <v>1697</v>
       </c>
       <c r="G4" s="0">
-        <v>9193</v>
+        <v>7331</v>
       </c>
       <c r="H4" s="0">
-        <v>1441</v>
+        <v>3303</v>
       </c>
       <c r="I4" s="0">
-        <v>1771</v>
+        <v>683</v>
       </c>
     </row>
     <row r="5">
@@ -1248,28 +1248,28 @@
         <v>4</v>
       </c>
       <c r="B5" s="0">
-        <v>0.71895973154362414</v>
+        <v>0.822212183789365</v>
       </c>
       <c r="C5" s="0">
-        <v>0.1665071770334928</v>
+        <v>0.21843971631205675</v>
       </c>
       <c r="D5" s="0">
-        <v>0.10609756097560975</v>
+        <v>0.16041666666666668</v>
       </c>
       <c r="E5" s="0">
-        <v>0.38666666666666666</v>
+        <v>0.34222222222222221</v>
       </c>
       <c r="F5" s="0">
-        <v>435</v>
+        <v>385</v>
       </c>
       <c r="G5" s="0">
-        <v>10706</v>
+        <v>12356</v>
       </c>
       <c r="H5" s="0">
-        <v>3665</v>
+        <v>2015</v>
       </c>
       <c r="I5" s="0">
-        <v>690</v>
+        <v>740</v>
       </c>
     </row>
     <row r="6">
@@ -1277,28 +1277,28 @@
         <v>5</v>
       </c>
       <c r="B6" s="0">
-        <v>0.56125108601216334</v>
+        <v>0.61751685904596421</v>
       </c>
       <c r="C6" s="0">
-        <v>0.202331703647988</v>
+        <v>0.44789489399820842</v>
       </c>
       <c r="D6" s="0">
-        <v>0.17467532467532468</v>
+        <v>0.33632286995515698</v>
       </c>
       <c r="E6" s="0">
-        <v>0.24039320822162646</v>
+        <v>0.67024128686327078</v>
       </c>
       <c r="F6" s="0">
-        <v>1345</v>
+        <v>3750</v>
       </c>
       <c r="G6" s="0">
-        <v>12221</v>
+        <v>11176</v>
       </c>
       <c r="H6" s="0">
-        <v>6355</v>
+        <v>7400</v>
       </c>
       <c r="I6" s="0">
-        <v>4250</v>
+        <v>1845</v>
       </c>
     </row>
     <row r="7">
@@ -1306,28 +1306,28 @@
         <v>6</v>
       </c>
       <c r="B7" s="0">
-        <v>0.6824030817146135</v>
+        <v>0.65125809359888531</v>
       </c>
       <c r="C7" s="0">
-        <v>0.47314751869476551</v>
+        <v>0.40112596762843067</v>
       </c>
       <c r="D7" s="0">
-        <v>0.40941176470588236</v>
+        <v>0.35625000000000001</v>
       </c>
       <c r="E7" s="0">
-        <v>0.56038647342995174</v>
+        <v>0.45893719806763283</v>
       </c>
       <c r="F7" s="0">
-        <v>1740</v>
+        <v>1425</v>
       </c>
       <c r="G7" s="0">
-        <v>6586</v>
+        <v>6521</v>
       </c>
       <c r="H7" s="0">
-        <v>2510</v>
+        <v>2575</v>
       </c>
       <c r="I7" s="0">
-        <v>1365</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="8">
@@ -1335,28 +1335,28 @@
         <v>7</v>
       </c>
       <c r="B8" s="0">
-        <v>0.81106861434956912</v>
+        <v>0.88618036035205749</v>
       </c>
       <c r="C8" s="0">
-        <v>0.046511627906976744</v>
+        <v>0.25151515151515152</v>
       </c>
       <c r="D8" s="0">
-        <v>0.036363636363636362</v>
+        <v>0.23714285714285716</v>
       </c>
       <c r="E8" s="0">
-        <v>0.064516129032258063</v>
+        <v>0.26774193548387099</v>
       </c>
       <c r="F8" s="0">
-        <v>100</v>
+        <v>415</v>
       </c>
       <c r="G8" s="0">
-        <v>17501</v>
+        <v>18816</v>
       </c>
       <c r="H8" s="0">
-        <v>2650</v>
+        <v>1335</v>
       </c>
       <c r="I8" s="0">
-        <v>1450</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="9">
@@ -1364,7 +1364,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="0">
-        <v>0.9278521295610096</v>
+        <v>0.93003182353197611</v>
       </c>
       <c r="C9" s="0">
         <v>0</v>
@@ -1379,10 +1379,10 @@
         <v>0</v>
       </c>
       <c r="G9" s="0">
-        <v>21284</v>
+        <v>21334</v>
       </c>
       <c r="H9" s="0">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="I9" s="0">
         <v>1405</v>
@@ -1393,28 +1393,28 @@
         <v>9</v>
       </c>
       <c r="B10" s="0">
-        <v>0.8708501570210857</v>
+        <v>0.89821668909825036</v>
       </c>
       <c r="C10" s="0">
-        <v>0.073239436619718309</v>
+        <v>0.52047556142668427</v>
       </c>
       <c r="D10" s="0">
-        <v>0.082727272727272733</v>
+        <v>0.41041666666666665</v>
       </c>
       <c r="E10" s="0">
-        <v>0.065703971119133578</v>
+        <v>0.71119133574007221</v>
       </c>
       <c r="F10" s="0">
-        <v>91</v>
+        <v>985</v>
       </c>
       <c r="G10" s="0">
-        <v>15438</v>
+        <v>15032</v>
       </c>
       <c r="H10" s="0">
-        <v>1009</v>
+        <v>1415</v>
       </c>
       <c r="I10" s="0">
-        <v>1294</v>
+        <v>400</v>
       </c>
     </row>
     <row r="11">
@@ -1422,28 +1422,28 @@
         <v>10</v>
       </c>
       <c r="B11" s="0">
-        <v>0.83188619988915569</v>
+        <v>0.82264917790504344</v>
       </c>
       <c r="C11" s="0">
-        <v>0.26612903225806456</v>
+        <v>0.26996197718631182</v>
       </c>
       <c r="D11" s="0">
-        <v>0.26400000000000001</v>
+        <v>0.25357142857142856</v>
       </c>
       <c r="E11" s="0">
-        <v>0.26829268292682928</v>
+        <v>0.2886178861788618</v>
       </c>
       <c r="F11" s="0">
-        <v>330</v>
+        <v>355</v>
       </c>
       <c r="G11" s="0">
-        <v>8676</v>
+        <v>8551</v>
       </c>
       <c r="H11" s="0">
-        <v>920</v>
+        <v>1045</v>
       </c>
       <c r="I11" s="0">
-        <v>900</v>
+        <v>875</v>
       </c>
     </row>
     <row r="12">
@@ -1451,28 +1451,28 @@
         <v>11</v>
       </c>
       <c r="B12" s="0">
-        <v>0.71462633186796809</v>
+        <v>0.6587437597794501</v>
       </c>
       <c r="C12" s="0">
-        <v>0.18683651804670912</v>
+        <v>0.19081272084805651</v>
       </c>
       <c r="D12" s="0">
-        <v>0.13333333333333333</v>
+        <v>0.12705882352941175</v>
       </c>
       <c r="E12" s="0">
-        <v>0.31205673758865249</v>
+        <v>0.38297872340425532</v>
       </c>
       <c r="F12" s="0">
-        <v>440</v>
+        <v>540</v>
       </c>
       <c r="G12" s="0">
-        <v>9151</v>
+        <v>8301</v>
       </c>
       <c r="H12" s="0">
-        <v>2860</v>
+        <v>3710</v>
       </c>
       <c r="I12" s="0">
-        <v>970</v>
+        <v>870</v>
       </c>
     </row>
     <row r="13">
@@ -1480,28 +1480,28 @@
         <v>12</v>
       </c>
       <c r="B13" s="0">
-        <v>0.81799832962138086</v>
+        <v>0.80992483296213813</v>
       </c>
       <c r="C13" s="0">
-        <v>0</v>
+        <v>0.10897226753670472</v>
       </c>
       <c r="D13" s="0">
-        <v>0</v>
+        <v>0.11517241379310345</v>
       </c>
       <c r="E13" s="0">
-        <v>0</v>
+        <v>0.10340557275541795</v>
       </c>
       <c r="F13" s="0">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="G13" s="0">
-        <v>11753</v>
+        <v>11470</v>
       </c>
       <c r="H13" s="0">
-        <v>1000</v>
+        <v>1283</v>
       </c>
       <c r="I13" s="0">
-        <v>1615</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="14">
@@ -1509,28 +1509,28 @@
         <v>13</v>
       </c>
       <c r="B14" s="0">
-        <v>0.75082001904560369</v>
+        <v>0.67992804994180511</v>
       </c>
       <c r="C14" s="0">
-        <v>0.21105527638190952</v>
+        <v>0.28571428571428575</v>
       </c>
       <c r="D14" s="0">
-        <v>0.17499999999999999</v>
+        <v>0.19836065573770492</v>
       </c>
       <c r="E14" s="0">
-        <v>0.26582278481012656</v>
+        <v>0.51054852320675104</v>
       </c>
       <c r="F14" s="0">
-        <v>315</v>
+        <v>605</v>
       </c>
       <c r="G14" s="0">
-        <v>6781</v>
+        <v>5821</v>
       </c>
       <c r="H14" s="0">
-        <v>1485</v>
+        <v>2445</v>
       </c>
       <c r="I14" s="0">
-        <v>870</v>
+        <v>580</v>
       </c>
     </row>
     <row r="15">
@@ -1538,28 +1538,28 @@
         <v>14</v>
       </c>
       <c r="B15" s="0">
-        <v>0.7719366061074604</v>
+        <v>0.64952969978095609</v>
       </c>
       <c r="C15" s="0">
-        <v>0.34926470588235292</v>
+        <v>0.18072289156626506</v>
       </c>
       <c r="D15" s="0">
-        <v>0.296875</v>
+        <v>0.13636363636363635</v>
       </c>
       <c r="E15" s="0">
-        <v>0.42410714285714285</v>
+        <v>0.26785714285714285</v>
       </c>
       <c r="F15" s="0">
-        <v>475</v>
+        <v>300</v>
       </c>
       <c r="G15" s="0">
-        <v>5516</v>
+        <v>4741</v>
       </c>
       <c r="H15" s="0">
-        <v>1125</v>
+        <v>1900</v>
       </c>
       <c r="I15" s="0">
-        <v>645</v>
+        <v>820</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated optimisation scripts to to be consistent with data loading in evaluator scripts
</commit_message>
<xml_diff>
--- a/mstraczkiewicz/MStraPlots_FreeLiving/FreeLiving_MStra_Results.xlsx
+++ b/mstraczkiewicz/MStraPlots_FreeLiving/FreeLiving_MStra_Results.xlsx
@@ -9,6 +9,7 @@
     <sheet name="All" sheetId="2" r:id="rId3"/>
     <sheet name="By_Subject" sheetId="3" r:id="rId5"/>
     <sheet name="All_Files" sheetId="4" r:id="rId6"/>
+    <sheet name="Data_Quality" sheetId="5" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
@@ -16,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="841" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="922" uniqueCount="51">
   <si>
     <t>Subject</t>
   </si>
@@ -112,6 +113,63 @@
   </si>
   <si>
     <t>sum_FN</t>
+  </si>
+  <si>
+    <t>File</t>
+  </si>
+  <si>
+    <t>Device2_sub12_annotated.csv</t>
+  </si>
+  <si>
+    <t>Device2_sub13_annotated.csv</t>
+  </si>
+  <si>
+    <t>Device2_sub14_annotated.csv</t>
+  </si>
+  <si>
+    <t>Device2_sub16_annotated.csv</t>
+  </si>
+  <si>
+    <t>Device2_sub17_annotated.csv</t>
+  </si>
+  <si>
+    <t>Device2_sub1_annotated.csv</t>
+  </si>
+  <si>
+    <t>Device2_sub2_annotated.csv</t>
+  </si>
+  <si>
+    <t>Device2_sub3_annotated.csv</t>
+  </si>
+  <si>
+    <t>Device2_sub4_annotated.csv</t>
+  </si>
+  <si>
+    <t>Device2_sub5_annotated.csv</t>
+  </si>
+  <si>
+    <t>Device2_sub6_annotated.csv</t>
+  </si>
+  <si>
+    <t>Device2_sub7_annotated.csv</t>
+  </si>
+  <si>
+    <t>Device2_sub8_annotated.csv</t>
+  </si>
+  <si>
+    <t>Device2_sub9_annotated.csv</t>
+  </si>
+  <si>
+    <t>TotalSec</t>
+  </si>
+  <si>
+    <t>ValidSec</t>
+  </si>
+  <si>
+    <t>RemovedSec</t>
+  </si>
+  <si>
+    <t>RemovedPct</t>
   </si>
 </sst>
 </file>
@@ -673,7 +731,7 @@
         <v>2575</v>
       </c>
       <c r="E2" s="0">
-        <v>6521</v>
+        <v>6520</v>
       </c>
       <c r="F2" s="0">
         <v>1680</v>
@@ -685,7 +743,7 @@
         <v>0.45893719806763283</v>
       </c>
       <c r="I2" s="0">
-        <v>0.65125809359888531</v>
+        <v>0.65122950819672132</v>
       </c>
       <c r="J2" s="0">
         <v>0.40112596762843067</v>
@@ -705,7 +763,7 @@
         <v>4185</v>
       </c>
       <c r="E3" s="0">
-        <v>17651</v>
+        <v>17650</v>
       </c>
       <c r="F3" s="0">
         <v>185</v>
@@ -717,7 +775,7 @@
         <v>0.78235294117647058</v>
       </c>
       <c r="I3" s="0">
-        <v>0.80737018425460638</v>
+        <v>0.80736169274851222</v>
       </c>
       <c r="J3" s="0">
         <v>0.23333333333333334</v>
@@ -737,7 +795,7 @@
         <v>3705</v>
       </c>
       <c r="E4" s="0">
-        <v>9671</v>
+        <v>9670</v>
       </c>
       <c r="F4" s="0">
         <v>605</v>
@@ -749,7 +807,7 @@
         <v>0.74791666666666667</v>
       </c>
       <c r="I4" s="0">
-        <v>0.72680020283975655</v>
+        <v>0.7267828843106181</v>
       </c>
       <c r="J4" s="0">
         <v>0.45443037974683548</v>
@@ -769,7 +827,7 @@
         <v>3303</v>
       </c>
       <c r="E5" s="0">
-        <v>7331</v>
+        <v>7330</v>
       </c>
       <c r="F5" s="0">
         <v>683</v>
@@ -781,7 +839,7 @@
         <v>0.71302521008403363</v>
       </c>
       <c r="I5" s="0">
-        <v>0.69371446134931614</v>
+        <v>0.69369092446015523</v>
       </c>
       <c r="J5" s="0">
         <v>0.45989159891598913</v>
@@ -801,7 +859,7 @@
         <v>2015</v>
       </c>
       <c r="E6" s="0">
-        <v>12356</v>
+        <v>12355</v>
       </c>
       <c r="F6" s="0">
         <v>740</v>
@@ -813,7 +871,7 @@
         <v>0.34222222222222221</v>
       </c>
       <c r="I6" s="0">
-        <v>0.822212183789365</v>
+        <v>0.82220070990642147</v>
       </c>
       <c r="J6" s="0">
         <v>0.21843971631205675</v>
@@ -833,7 +891,7 @@
         <v>7400</v>
       </c>
       <c r="E7" s="0">
-        <v>11176</v>
+        <v>11175</v>
       </c>
       <c r="F7" s="0">
         <v>1845</v>
@@ -845,7 +903,7 @@
         <v>0.67024128686327078</v>
       </c>
       <c r="I7" s="0">
-        <v>0.61751685904596421</v>
+        <v>0.61750103434009107</v>
       </c>
       <c r="J7" s="0">
         <v>0.44789489399820842</v>
@@ -865,7 +923,7 @@
         <v>1335</v>
       </c>
       <c r="E8" s="0">
-        <v>18816</v>
+        <v>18815</v>
       </c>
       <c r="F8" s="0">
         <v>1135</v>
@@ -877,7 +935,7 @@
         <v>0.26774193548387099</v>
       </c>
       <c r="I8" s="0">
-        <v>0.88618036035205749</v>
+        <v>0.88617511520737324</v>
       </c>
       <c r="J8" s="0">
         <v>0.25151515151515152</v>
@@ -897,7 +955,7 @@
         <v>200</v>
       </c>
       <c r="E9" s="0">
-        <v>21334</v>
+        <v>21333</v>
       </c>
       <c r="F9" s="0">
         <v>1405</v>
@@ -909,7 +967,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="0">
-        <v>0.93003182353197611</v>
+        <v>0.93002877321475286</v>
       </c>
       <c r="J9" s="0">
         <v>0</v>
@@ -929,7 +987,7 @@
         <v>1415</v>
       </c>
       <c r="E10" s="0">
-        <v>15032</v>
+        <v>15031</v>
       </c>
       <c r="F10" s="0">
         <v>400</v>
@@ -941,7 +999,7 @@
         <v>0.71119133574007221</v>
       </c>
       <c r="I10" s="0">
-        <v>0.89821668909825036</v>
+        <v>0.89821098087600248</v>
       </c>
       <c r="J10" s="0">
         <v>0.52047556142668427</v>
@@ -961,7 +1019,7 @@
         <v>1045</v>
       </c>
       <c r="E11" s="0">
-        <v>8551</v>
+        <v>8550</v>
       </c>
       <c r="F11" s="0">
         <v>875</v>
@@ -973,7 +1031,7 @@
         <v>0.2886178861788618</v>
       </c>
       <c r="I11" s="0">
-        <v>0.82264917790504344</v>
+        <v>0.82263279445727477</v>
       </c>
       <c r="J11" s="0">
         <v>0.26996197718631182</v>
@@ -993,7 +1051,7 @@
         <v>3710</v>
       </c>
       <c r="E12" s="0">
-        <v>8301</v>
+        <v>8300</v>
       </c>
       <c r="F12" s="0">
         <v>870</v>
@@ -1005,7 +1063,7 @@
         <v>0.38297872340425532</v>
       </c>
       <c r="I12" s="0">
-        <v>0.6587437597794501</v>
+        <v>0.6587183308494784</v>
       </c>
       <c r="J12" s="0">
         <v>0.19081272084805651</v>
@@ -1025,7 +1083,7 @@
         <v>1283</v>
       </c>
       <c r="E13" s="0">
-        <v>11470</v>
+        <v>11469</v>
       </c>
       <c r="F13" s="0">
         <v>1448</v>
@@ -1037,7 +1095,7 @@
         <v>0.10340557275541795</v>
       </c>
       <c r="I13" s="0">
-        <v>0.80992483296213813</v>
+        <v>0.80991160297904918</v>
       </c>
       <c r="J13" s="0">
         <v>0.10897226753670472</v>
@@ -1057,7 +1115,7 @@
         <v>2445</v>
       </c>
       <c r="E14" s="0">
-        <v>5821</v>
+        <v>5820</v>
       </c>
       <c r="F14" s="0">
         <v>580</v>
@@ -1069,7 +1127,7 @@
         <v>0.51054852320675104</v>
       </c>
       <c r="I14" s="0">
-        <v>0.67992804994180511</v>
+        <v>0.67989417989417988</v>
       </c>
       <c r="J14" s="0">
         <v>0.28571428571428575</v>
@@ -1086,25 +1144,25 @@
         <v>300</v>
       </c>
       <c r="D15" s="0">
-        <v>1900</v>
+        <v>1950</v>
       </c>
       <c r="E15" s="0">
-        <v>4741</v>
+        <v>4690</v>
       </c>
       <c r="F15" s="0">
         <v>820</v>
       </c>
       <c r="G15" s="0">
-        <v>0.13636363636363635</v>
+        <v>0.13333333333333333</v>
       </c>
       <c r="H15" s="0">
         <v>0.26785714285714285</v>
       </c>
       <c r="I15" s="0">
-        <v>0.64952969978095609</v>
+        <v>0.64304123711340211</v>
       </c>
       <c r="J15" s="0">
-        <v>0.18072289156626506</v>
+        <v>0.17804154302670622</v>
       </c>
     </row>
   </sheetData>
@@ -1161,7 +1219,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="0">
-        <v>0.80737018425460638</v>
+        <v>0.80736169274851222</v>
       </c>
       <c r="C2" s="0">
         <v>0.23333333333333334</v>
@@ -1176,7 +1234,7 @@
         <v>665</v>
       </c>
       <c r="G2" s="0">
-        <v>17651</v>
+        <v>17650</v>
       </c>
       <c r="H2" s="0">
         <v>4185</v>
@@ -1190,7 +1248,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="0">
-        <v>0.72680020283975655</v>
+        <v>0.7267828843106181</v>
       </c>
       <c r="C3" s="0">
         <v>0.45443037974683548</v>
@@ -1205,7 +1263,7 @@
         <v>1795</v>
       </c>
       <c r="G3" s="0">
-        <v>9671</v>
+        <v>9670</v>
       </c>
       <c r="H3" s="0">
         <v>3705</v>
@@ -1219,7 +1277,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="0">
-        <v>0.69371446134931614</v>
+        <v>0.69369092446015523</v>
       </c>
       <c r="C4" s="0">
         <v>0.45989159891598913</v>
@@ -1234,7 +1292,7 @@
         <v>1697</v>
       </c>
       <c r="G4" s="0">
-        <v>7331</v>
+        <v>7330</v>
       </c>
       <c r="H4" s="0">
         <v>3303</v>
@@ -1248,7 +1306,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="0">
-        <v>0.822212183789365</v>
+        <v>0.82220070990642147</v>
       </c>
       <c r="C5" s="0">
         <v>0.21843971631205675</v>
@@ -1263,7 +1321,7 @@
         <v>385</v>
       </c>
       <c r="G5" s="0">
-        <v>12356</v>
+        <v>12355</v>
       </c>
       <c r="H5" s="0">
         <v>2015</v>
@@ -1277,7 +1335,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="0">
-        <v>0.61751685904596421</v>
+        <v>0.61750103434009107</v>
       </c>
       <c r="C6" s="0">
         <v>0.44789489399820842</v>
@@ -1292,7 +1350,7 @@
         <v>3750</v>
       </c>
       <c r="G6" s="0">
-        <v>11176</v>
+        <v>11175</v>
       </c>
       <c r="H6" s="0">
         <v>7400</v>
@@ -1306,7 +1364,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="0">
-        <v>0.65125809359888531</v>
+        <v>0.65122950819672132</v>
       </c>
       <c r="C7" s="0">
         <v>0.40112596762843067</v>
@@ -1321,7 +1379,7 @@
         <v>1425</v>
       </c>
       <c r="G7" s="0">
-        <v>6521</v>
+        <v>6520</v>
       </c>
       <c r="H7" s="0">
         <v>2575</v>
@@ -1335,7 +1393,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="0">
-        <v>0.88618036035205749</v>
+        <v>0.88617511520737324</v>
       </c>
       <c r="C8" s="0">
         <v>0.25151515151515152</v>
@@ -1350,7 +1408,7 @@
         <v>415</v>
       </c>
       <c r="G8" s="0">
-        <v>18816</v>
+        <v>18815</v>
       </c>
       <c r="H8" s="0">
         <v>1335</v>
@@ -1364,7 +1422,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="0">
-        <v>0.93003182353197611</v>
+        <v>0.93002877321475286</v>
       </c>
       <c r="C9" s="0">
         <v>0</v>
@@ -1379,7 +1437,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="0">
-        <v>21334</v>
+        <v>21333</v>
       </c>
       <c r="H9" s="0">
         <v>200</v>
@@ -1393,7 +1451,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="0">
-        <v>0.89821668909825036</v>
+        <v>0.89821098087600248</v>
       </c>
       <c r="C10" s="0">
         <v>0.52047556142668427</v>
@@ -1408,7 +1466,7 @@
         <v>985</v>
       </c>
       <c r="G10" s="0">
-        <v>15032</v>
+        <v>15031</v>
       </c>
       <c r="H10" s="0">
         <v>1415</v>
@@ -1422,7 +1480,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="0">
-        <v>0.82264917790504344</v>
+        <v>0.82263279445727477</v>
       </c>
       <c r="C11" s="0">
         <v>0.26996197718631182</v>
@@ -1437,7 +1495,7 @@
         <v>355</v>
       </c>
       <c r="G11" s="0">
-        <v>8551</v>
+        <v>8550</v>
       </c>
       <c r="H11" s="0">
         <v>1045</v>
@@ -1451,7 +1509,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="0">
-        <v>0.6587437597794501</v>
+        <v>0.6587183308494784</v>
       </c>
       <c r="C12" s="0">
         <v>0.19081272084805651</v>
@@ -1466,7 +1524,7 @@
         <v>540</v>
       </c>
       <c r="G12" s="0">
-        <v>8301</v>
+        <v>8300</v>
       </c>
       <c r="H12" s="0">
         <v>3710</v>
@@ -1480,7 +1538,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="0">
-        <v>0.80992483296213813</v>
+        <v>0.80991160297904918</v>
       </c>
       <c r="C13" s="0">
         <v>0.10897226753670472</v>
@@ -1495,7 +1553,7 @@
         <v>167</v>
       </c>
       <c r="G13" s="0">
-        <v>11470</v>
+        <v>11469</v>
       </c>
       <c r="H13" s="0">
         <v>1283</v>
@@ -1509,7 +1567,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="0">
-        <v>0.67992804994180511</v>
+        <v>0.67989417989417988</v>
       </c>
       <c r="C14" s="0">
         <v>0.28571428571428575</v>
@@ -1524,7 +1582,7 @@
         <v>605</v>
       </c>
       <c r="G14" s="0">
-        <v>5821</v>
+        <v>5820</v>
       </c>
       <c r="H14" s="0">
         <v>2445</v>
@@ -1538,13 +1596,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="0">
-        <v>0.64952969978095609</v>
+        <v>0.64304123711340211</v>
       </c>
       <c r="C15" s="0">
-        <v>0.18072289156626506</v>
+        <v>0.17804154302670622</v>
       </c>
       <c r="D15" s="0">
-        <v>0.13636363636363635</v>
+        <v>0.13333333333333333</v>
       </c>
       <c r="E15" s="0">
         <v>0.26785714285714285</v>
@@ -1553,13 +1611,330 @@
         <v>300</v>
       </c>
       <c r="G15" s="0">
-        <v>4741</v>
+        <v>4690</v>
       </c>
       <c r="H15" s="0">
-        <v>1900</v>
+        <v>1950</v>
       </c>
       <c r="I15" s="0">
         <v>820</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="6.88671875" customWidth="true"/>
+    <col min="2" max="2" width="25.77734375" customWidth="true"/>
+    <col min="3" max="3" width="8" customWidth="true"/>
+    <col min="4" max="4" width="7.77734375" customWidth="true"/>
+    <col min="5" max="5" width="11.44140625" customWidth="true"/>
+    <col min="6" max="6" width="12.5546875" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="0">
+        <v>455.68000000000001</v>
+      </c>
+      <c r="D2" s="0">
+        <v>453.69999999999999</v>
+      </c>
+      <c r="E2" s="0">
+        <v>1.9800000000000182</v>
+      </c>
+      <c r="F2" s="0">
+        <v>0.43451544943820625</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="0">
+        <v>317.48000000000002</v>
+      </c>
+      <c r="D3" s="0">
+        <v>315.5</v>
+      </c>
+      <c r="E3" s="0">
+        <v>1.9800000000000182</v>
+      </c>
+      <c r="F3" s="0">
+        <v>0.62366133299735982</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="0">
+        <v>262.24000000000001</v>
+      </c>
+      <c r="D4" s="0">
+        <v>260.25999999999999</v>
+      </c>
+      <c r="E4" s="0">
+        <v>1.9800000000000182</v>
+      </c>
+      <c r="F4" s="0">
+        <v>0.75503355704698683</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="0">
+        <v>311.88</v>
+      </c>
+      <c r="D5" s="0">
+        <v>309.89999999999998</v>
+      </c>
+      <c r="E5" s="0">
+        <v>1.9800000000000182</v>
+      </c>
+      <c r="F5" s="0">
+        <v>0.6348595613697634</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="0">
+        <v>485.38</v>
+      </c>
+      <c r="D6" s="0">
+        <v>483.39999999999998</v>
+      </c>
+      <c r="E6" s="0">
+        <v>1.9800000000000182</v>
+      </c>
+      <c r="F6" s="0">
+        <v>0.40792780913923488</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="0">
+        <v>245.97999999999999</v>
+      </c>
+      <c r="D7" s="0">
+        <v>244</v>
+      </c>
+      <c r="E7" s="0">
+        <v>1.9799999999999898</v>
+      </c>
+      <c r="F7" s="0">
+        <v>0.80494349134075527</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="0">
+        <v>435.98000000000002</v>
+      </c>
+      <c r="D8" s="0">
+        <v>434</v>
+      </c>
+      <c r="E8" s="0">
+        <v>1.9800000000000182</v>
+      </c>
+      <c r="F8" s="0">
+        <v>0.45414927290243085</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="0">
+        <v>460.74000000000001</v>
+      </c>
+      <c r="D9" s="0">
+        <v>458.75999999999999</v>
+      </c>
+      <c r="E9" s="0">
+        <v>1.9800000000000182</v>
+      </c>
+      <c r="F9" s="0">
+        <v>0.42974345617919396</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="0">
+        <v>358.60000000000002</v>
+      </c>
+      <c r="D10" s="0">
+        <v>356.62</v>
+      </c>
+      <c r="E10" s="0">
+        <v>1.9800000000000182</v>
+      </c>
+      <c r="F10" s="0">
+        <v>0.55214723926380871</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="0">
+        <v>218.47999999999999</v>
+      </c>
+      <c r="D11" s="0">
+        <v>216.5</v>
+      </c>
+      <c r="E11" s="0">
+        <v>1.9799999999999898</v>
+      </c>
+      <c r="F11" s="0">
+        <v>0.90626144269497888</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="0">
+        <v>270.38</v>
+      </c>
+      <c r="D12" s="0">
+        <v>268.39999999999998</v>
+      </c>
+      <c r="E12" s="0">
+        <v>1.9800000000000182</v>
+      </c>
+      <c r="F12" s="0">
+        <v>0.73230268510985219</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="0">
+        <v>289.31999999999999</v>
+      </c>
+      <c r="D13" s="0">
+        <v>287.33999999999997</v>
+      </c>
+      <c r="E13" s="0">
+        <v>1.9800000000000182</v>
+      </c>
+      <c r="F13" s="0">
+        <v>0.68436333471589184</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="0">
+        <v>190.97999999999999</v>
+      </c>
+      <c r="D14" s="0">
+        <v>189</v>
+      </c>
+      <c r="E14" s="0">
+        <v>1.9799999999999898</v>
+      </c>
+      <c r="F14" s="0">
+        <v>1.0367577756833124</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="0">
+        <v>157.18000000000001</v>
+      </c>
+      <c r="D15" s="0">
+        <v>155.19999999999999</v>
+      </c>
+      <c r="E15" s="0">
+        <v>1.9800000000000182</v>
+      </c>
+      <c r="F15" s="0">
+        <v>1.2597022521949472</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed print statements to show quantity of faulty data as well as final data quality review
</commit_message>
<xml_diff>
--- a/mstraczkiewicz/MStraPlots_FreeLiving/FreeLiving_MStra_Results.xlsx
+++ b/mstraczkiewicz/MStraPlots_FreeLiving/FreeLiving_MStra_Results.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="922" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="1039" uniqueCount="55">
   <si>
     <t>Subject</t>
   </si>
@@ -170,6 +170,18 @@
   </si>
   <si>
     <t>RemovedPct</t>
+  </si>
+  <si>
+    <t>TotalRawRows</t>
+  </si>
+  <si>
+    <t>FaultyRowsRemoved</t>
+  </si>
+  <si>
+    <t>TotalCleanedSec</t>
+  </si>
+  <si>
+    <t>EvaluableSec</t>
   </si>
 </sst>
 </file>
@@ -1626,15 +1638,17 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.88671875" customWidth="true"/>
     <col min="2" max="2" width="25.77734375" customWidth="true"/>
-    <col min="3" max="3" width="8" customWidth="true"/>
-    <col min="4" max="4" width="7.77734375" customWidth="true"/>
-    <col min="5" max="5" width="11.44140625" customWidth="true"/>
-    <col min="6" max="6" width="12.5546875" customWidth="true"/>
+    <col min="3" max="3" width="13.21875" customWidth="true"/>
+    <col min="4" max="4" width="18" customWidth="true"/>
+    <col min="5" max="5" width="14.5546875" customWidth="true"/>
+    <col min="6" max="6" width="11.5546875" customWidth="true"/>
+    <col min="7" max="7" width="11.44140625" customWidth="true"/>
+    <col min="8" max="8" width="12.5546875" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1645,15 +1659,21 @@
         <v>32</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E1" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1" s="0" t="s">
         <v>49</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="H1" s="0" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1665,15 +1685,21 @@
         <v>33</v>
       </c>
       <c r="C2" s="0">
+        <v>22785</v>
+      </c>
+      <c r="D2" s="0">
+        <v>0</v>
+      </c>
+      <c r="E2" s="0">
         <v>455.68000000000001</v>
       </c>
-      <c r="D2" s="0">
+      <c r="F2" s="0">
         <v>453.69999999999999</v>
       </c>
-      <c r="E2" s="0">
+      <c r="G2" s="0">
         <v>1.9800000000000182</v>
       </c>
-      <c r="F2" s="0">
+      <c r="H2" s="0">
         <v>0.43451544943820625</v>
       </c>
     </row>
@@ -1685,15 +1711,21 @@
         <v>34</v>
       </c>
       <c r="C3" s="0">
+        <v>15875</v>
+      </c>
+      <c r="D3" s="0">
+        <v>0</v>
+      </c>
+      <c r="E3" s="0">
         <v>317.48000000000002</v>
       </c>
-      <c r="D3" s="0">
+      <c r="F3" s="0">
         <v>315.5</v>
       </c>
-      <c r="E3" s="0">
+      <c r="G3" s="0">
         <v>1.9800000000000182</v>
       </c>
-      <c r="F3" s="0">
+      <c r="H3" s="0">
         <v>0.62366133299735982</v>
       </c>
     </row>
@@ -1705,15 +1737,21 @@
         <v>35</v>
       </c>
       <c r="C4" s="0">
+        <v>13113</v>
+      </c>
+      <c r="D4" s="0">
+        <v>0</v>
+      </c>
+      <c r="E4" s="0">
         <v>262.24000000000001</v>
       </c>
-      <c r="D4" s="0">
+      <c r="F4" s="0">
         <v>260.25999999999999</v>
       </c>
-      <c r="E4" s="0">
+      <c r="G4" s="0">
         <v>1.9800000000000182</v>
       </c>
-      <c r="F4" s="0">
+      <c r="H4" s="0">
         <v>0.75503355704698683</v>
       </c>
     </row>
@@ -1725,15 +1763,21 @@
         <v>36</v>
       </c>
       <c r="C5" s="0">
+        <v>15595</v>
+      </c>
+      <c r="D5" s="0">
+        <v>0</v>
+      </c>
+      <c r="E5" s="0">
         <v>311.88</v>
       </c>
-      <c r="D5" s="0">
+      <c r="F5" s="0">
         <v>309.89999999999998</v>
       </c>
-      <c r="E5" s="0">
+      <c r="G5" s="0">
         <v>1.9800000000000182</v>
       </c>
-      <c r="F5" s="0">
+      <c r="H5" s="0">
         <v>0.6348595613697634</v>
       </c>
     </row>
@@ -1745,15 +1789,21 @@
         <v>37</v>
       </c>
       <c r="C6" s="0">
+        <v>24270</v>
+      </c>
+      <c r="D6" s="0">
+        <v>0</v>
+      </c>
+      <c r="E6" s="0">
         <v>485.38</v>
       </c>
-      <c r="D6" s="0">
+      <c r="F6" s="0">
         <v>483.39999999999998</v>
       </c>
-      <c r="E6" s="0">
+      <c r="G6" s="0">
         <v>1.9800000000000182</v>
       </c>
-      <c r="F6" s="0">
+      <c r="H6" s="0">
         <v>0.40792780913923488</v>
       </c>
     </row>
@@ -1765,15 +1815,21 @@
         <v>38</v>
       </c>
       <c r="C7" s="0">
+        <v>12300</v>
+      </c>
+      <c r="D7" s="0">
+        <v>0</v>
+      </c>
+      <c r="E7" s="0">
         <v>245.97999999999999</v>
       </c>
-      <c r="D7" s="0">
+      <c r="F7" s="0">
         <v>244</v>
       </c>
-      <c r="E7" s="0">
+      <c r="G7" s="0">
         <v>1.9799999999999898</v>
       </c>
-      <c r="F7" s="0">
+      <c r="H7" s="0">
         <v>0.80494349134075527</v>
       </c>
     </row>
@@ -1785,15 +1841,21 @@
         <v>39</v>
       </c>
       <c r="C8" s="0">
+        <v>21800</v>
+      </c>
+      <c r="D8" s="0">
+        <v>0</v>
+      </c>
+      <c r="E8" s="0">
         <v>435.98000000000002</v>
       </c>
-      <c r="D8" s="0">
+      <c r="F8" s="0">
         <v>434</v>
       </c>
-      <c r="E8" s="0">
+      <c r="G8" s="0">
         <v>1.9800000000000182</v>
       </c>
-      <c r="F8" s="0">
+      <c r="H8" s="0">
         <v>0.45414927290243085</v>
       </c>
     </row>
@@ -1805,15 +1867,21 @@
         <v>40</v>
       </c>
       <c r="C9" s="0">
+        <v>23038</v>
+      </c>
+      <c r="D9" s="0">
+        <v>0</v>
+      </c>
+      <c r="E9" s="0">
         <v>460.74000000000001</v>
       </c>
-      <c r="D9" s="0">
+      <c r="F9" s="0">
         <v>458.75999999999999</v>
       </c>
-      <c r="E9" s="0">
+      <c r="G9" s="0">
         <v>1.9800000000000182</v>
       </c>
-      <c r="F9" s="0">
+      <c r="H9" s="0">
         <v>0.42974345617919396</v>
       </c>
     </row>
@@ -1825,15 +1893,21 @@
         <v>41</v>
       </c>
       <c r="C10" s="0">
+        <v>17931</v>
+      </c>
+      <c r="D10" s="0">
+        <v>0</v>
+      </c>
+      <c r="E10" s="0">
         <v>358.60000000000002</v>
       </c>
-      <c r="D10" s="0">
+      <c r="F10" s="0">
         <v>356.62</v>
       </c>
-      <c r="E10" s="0">
+      <c r="G10" s="0">
         <v>1.9800000000000182</v>
       </c>
-      <c r="F10" s="0">
+      <c r="H10" s="0">
         <v>0.55214723926380871</v>
       </c>
     </row>
@@ -1845,15 +1919,21 @@
         <v>42</v>
       </c>
       <c r="C11" s="0">
+        <v>10925</v>
+      </c>
+      <c r="D11" s="0">
+        <v>0</v>
+      </c>
+      <c r="E11" s="0">
         <v>218.47999999999999</v>
       </c>
-      <c r="D11" s="0">
+      <c r="F11" s="0">
         <v>216.5</v>
       </c>
-      <c r="E11" s="0">
+      <c r="G11" s="0">
         <v>1.9799999999999898</v>
       </c>
-      <c r="F11" s="0">
+      <c r="H11" s="0">
         <v>0.90626144269497888</v>
       </c>
     </row>
@@ -1865,15 +1945,21 @@
         <v>43</v>
       </c>
       <c r="C12" s="0">
+        <v>13520</v>
+      </c>
+      <c r="D12" s="0">
+        <v>0</v>
+      </c>
+      <c r="E12" s="0">
         <v>270.38</v>
       </c>
-      <c r="D12" s="0">
+      <c r="F12" s="0">
         <v>268.39999999999998</v>
       </c>
-      <c r="E12" s="0">
+      <c r="G12" s="0">
         <v>1.9800000000000182</v>
       </c>
-      <c r="F12" s="0">
+      <c r="H12" s="0">
         <v>0.73230268510985219</v>
       </c>
     </row>
@@ -1885,15 +1971,21 @@
         <v>44</v>
       </c>
       <c r="C13" s="0">
+        <v>14467</v>
+      </c>
+      <c r="D13" s="0">
+        <v>0</v>
+      </c>
+      <c r="E13" s="0">
         <v>289.31999999999999</v>
       </c>
-      <c r="D13" s="0">
+      <c r="F13" s="0">
         <v>287.33999999999997</v>
       </c>
-      <c r="E13" s="0">
+      <c r="G13" s="0">
         <v>1.9800000000000182</v>
       </c>
-      <c r="F13" s="0">
+      <c r="H13" s="0">
         <v>0.68436333471589184</v>
       </c>
     </row>
@@ -1905,15 +1997,21 @@
         <v>45</v>
       </c>
       <c r="C14" s="0">
+        <v>9550</v>
+      </c>
+      <c r="D14" s="0">
+        <v>0</v>
+      </c>
+      <c r="E14" s="0">
         <v>190.97999999999999</v>
       </c>
-      <c r="D14" s="0">
+      <c r="F14" s="0">
         <v>189</v>
       </c>
-      <c r="E14" s="0">
+      <c r="G14" s="0">
         <v>1.9799999999999898</v>
       </c>
-      <c r="F14" s="0">
+      <c r="H14" s="0">
         <v>1.0367577756833124</v>
       </c>
     </row>
@@ -1925,15 +2023,21 @@
         <v>46</v>
       </c>
       <c r="C15" s="0">
+        <v>7860</v>
+      </c>
+      <c r="D15" s="0">
+        <v>0</v>
+      </c>
+      <c r="E15" s="0">
         <v>157.18000000000001</v>
       </c>
-      <c r="D15" s="0">
+      <c r="F15" s="0">
         <v>155.19999999999999</v>
       </c>
-      <c r="E15" s="0">
+      <c r="G15" s="0">
         <v>1.9800000000000182</v>
       </c>
-      <c r="F15" s="0">
+      <c r="H15" s="0">
         <v>1.2597022521949472</v>
       </c>
     </row>

</xml_diff>